<commit_message>
T1059.003 Windows Command Shell
</commit_message>
<xml_diff>
--- a/Windows Detection Rules/Master List.xlsx
+++ b/Windows Detection Rules/Master List.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Detection Engineering\Detection Rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Detection Engineering\Detection Rules\Windows Detection Rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE78097-1529-468A-9832-60DDA0CB3C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1272467-57EB-4CFD-9282-7EC08D13B935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,50 +25,23 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
   <si>
     <t>Technique</t>
   </si>
   <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>Expected event</t>
-  </si>
-  <si>
     <t>T1059.001</t>
   </si>
   <si>
     <t xml:space="preserve"> Atomic PowerShell test</t>
   </si>
   <si>
-    <t>Sysmon 1</t>
-  </si>
-  <si>
-    <t>Observed event</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Detection</t>
-  </si>
-  <si>
-    <t>Sentinel Ingestion</t>
-  </si>
-  <si>
-    <t>Alert</t>
-  </si>
-  <si>
     <t>False Postive</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
     <t>T1059.001 PowerShell</t>
   </si>
   <si>
@@ -199,6 +172,15 @@
   </si>
   <si>
     <t>Lateral Movement</t>
+  </si>
+  <si>
+    <t>Enabled</t>
+  </si>
+  <si>
+    <t>Atomic RedTeam Test Status</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -522,304 +504,274 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
     <col min="2" max="2" width="36.21875" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B29" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B34" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>